<commit_message>
Fix all model formulas, eliminate PDF clipping across all 4 pages, add candidate voice placeholders, and remove invented provenance
</commit_message>
<xml_diff>
--- a/cheerio/assignment/cheerio_cost_model.xlsx
+++ b/cheerio/assignment/cheerio_cost_model.xlsx
@@ -132,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -197,6 +197,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="169" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="169" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -576,7 +579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="78" customWidth="1" min="1" max="1"/>
@@ -584,7 +587,7 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="59" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -678,20 +681,20 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>QUERY_RATE</t>
+          <t>NEW_SIGNUPS</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Monthly Support Query Rate per Merchant</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="n">
-        <v>3.5</v>
+          <t>New Merchant Signups per Month</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>500</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Queries / biz / mo</t>
+          <t>Signups / mo</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -701,7 +704,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>5-7 queries in Month 1 onboarding; 1-2 in mature phase</t>
+          <t>Candidate estimate: 10% monthly onboarding cohort</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -713,30 +716,30 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>FX_USD_INR</t>
+          <t>QUERY_RATE</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>USD to INR Exchange Rate</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="n">
-        <v>84</v>
+          <t>Monthly Support Query Rate per Merchant</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>3.5</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>INR / USD</t>
+          <t>Queries / biz / mo</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Industry Benchmark</t>
+          <t>Stated Assumption</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>RBI Reference Exchange Rate (rbi.org.in)</t>
+          <t>Candidate estimate: 5-7 queries in onboarding; 1-2 in mature phase</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -748,30 +751,30 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>LLM_IN_PRICE</t>
+          <t>FX_USD_INR</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>GPT-4o-mini Input Token Price</t>
+          <t>USD to INR Exchange Rate</t>
         </is>
       </c>
       <c r="C8" s="9" t="n">
-        <v>0.15</v>
+        <v>84</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>USD / 1M tokens</t>
+          <t>INR / USD</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Verified API Pricing</t>
+          <t>Industry Benchmark</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>https://openai.com/api/pricing</t>
+          <t>RBI Reference Exchange Rate (rbi.org.in)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -783,16 +786,16 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>LLM_IN_CACHE</t>
+          <t>LLM_IN_PRICE</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>GPT-4o-mini Cached Input Token Price</t>
+          <t>GPT-4o-mini Input Token Price</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>0.075</v>
+        <v>0.15</v>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
@@ -806,7 +809,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>https://openai.com/api/pricing (50% cache hit discount)</t>
+          <t>https://openai.com/api/pricing</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -818,16 +821,16 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>LLM_OUT_PRICE</t>
+          <t>LLM_IN_CACHE</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>GPT-4o-mini Output Token Price</t>
+          <t>GPT-4o-mini Cached Input Token Price</t>
         </is>
       </c>
       <c r="C10" s="9" t="n">
-        <v>0.6</v>
+        <v>0.075</v>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
@@ -841,7 +844,7 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>https://openai.com/api/pricing</t>
+          <t>https://openai.com/api/pricing (50% cache hit discount)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -853,30 +856,30 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>TOKENS_IN</t>
+          <t>LLM_OUT_PRICE</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Average Input Tokens per Query Session</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>2500</v>
+          <t>GPT-4o-mini Output Token Price</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>0.6</v>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Tokens / query</t>
+          <t>USD / 1M tokens</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Stated Assumption</t>
+          <t>Verified API Pricing</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>System prompt (1k) + error payload (500) + 3 turns (1k)</t>
+          <t>https://openai.com/api/pricing</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -888,16 +891,16 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>TOKENS_OUT</t>
+          <t>TOKENS_IN</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Average Output Tokens per Query Session</t>
+          <t>Average Input Tokens per Query Session</t>
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>500</v>
+        <v>2500</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
@@ -911,7 +914,7 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>Structured diagnostic + JSON remediation payload</t>
+          <t>System prompt (1k) + error payload (500) + 3 turns (1k)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -923,30 +926,30 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>INFRA_OVERHEAD</t>
+          <t>TOKENS_OUT</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Serverless &amp; Redis Cache Buffer</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="n">
-        <v>0.1433</v>
+          <t>Average Output Tokens per Query Session</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>500</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>INR / query</t>
+          <t>Tokens / query</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Industry Benchmark</t>
+          <t>Stated Assumption</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>Cloudflare Workers &amp; Upstash Redis semantic cache</t>
+          <t>Structured diagnostic + JSON remediation payload</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -958,20 +961,20 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>AGENT_SALARY</t>
+          <t>INFRA_OVERHEAD</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Human Support Rep Monthly Salary</t>
-        </is>
-      </c>
-      <c r="C14" s="11" t="n">
-        <v>35000</v>
+          <t>Serverless &amp; Redis Cache Buffer</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>0.1433</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>INR / agent / mo</t>
+          <t>INR / query</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
@@ -981,7 +984,7 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>Glassdoor / AmbitionBox Indian B2B SaaS CS benchmark</t>
+          <t>Cloudflare Workers &amp; Upstash Redis semantic cache</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -993,30 +996,30 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>WORK_DAYS</t>
+          <t>AGENT_SALARY</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Working Days per Month</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>22</v>
+          <t>Human Support Rep Monthly Salary</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>35000</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Days / mo</t>
+          <t>INR / agent / mo</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Standard Work Week</t>
+          <t>Industry Benchmark</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>5-day work week standard</t>
+          <t>Glassdoor / AmbitionBox Indian B2B SaaS CS benchmark</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
@@ -1028,30 +1031,30 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>AGENT_TICKETS_DAY</t>
+          <t>WORK_DAYS</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Daily Ticket Handling Capacity per Rep</t>
+          <t>Working Days per Month</t>
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>Tickets / agent / day</t>
+          <t>Days / mo</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Stated Assumption</t>
+          <t>Standard Work Week</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>Assumes 12 mins per ticket across async chat / email</t>
+          <t>5-day work week standard</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -1063,20 +1066,20 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>BASE_DEFLECTION</t>
+          <t>AGENT_TICKETS_DAY</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Baseline Deflection Rate (Status Quo)</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="n">
-        <v>0.12</v>
+          <t>Daily Ticket Handling Capacity per Rep</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>40</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>% deflected</t>
+          <t>Tickets / agent / day</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
@@ -1086,7 +1089,7 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Static FAQ &amp; docs deflection prior to Co-Pilot</t>
+          <t>Assumes 12 mins per ticket across async chat / email</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
@@ -1098,16 +1101,16 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>TARGET_DEFLECTION</t>
+          <t>BASE_DEFLECTION</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Co-Pilot Target Deflection Rate (Base)</t>
+          <t>Baseline Deflection Rate (Status Quo)</t>
         </is>
       </c>
       <c r="C18" s="12" t="n">
-        <v>0.65</v>
+        <v>0.12</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
@@ -1116,12 +1119,12 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Stated Target</t>
+          <t>Stated Assumption</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Target across top 5 bottlenecks in 90 days</t>
+          <t>Static FAQ &amp; docs deflection prior to Co-Pilot</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1133,30 +1136,30 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>ZOCR_DAY90</t>
+          <t>TARGET_DEFLECTION</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Zero-Touch Onboarding Completion Rate</t>
+          <t>Co-Pilot Target Deflection Rate (Base)</t>
         </is>
       </c>
       <c r="C19" s="12" t="n">
-        <v>0.33</v>
+        <v>0.65</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>% rate</t>
+          <t>% deflected</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Realistic Target</t>
+          <t>Stated Target</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>Realistic 90-day trajectory: 22% baseline -&gt; 33%</t>
+          <t>Target across top technical bottlenecks in 90 days</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
@@ -1168,20 +1171,20 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>BUILD_COST</t>
+          <t>BASE_ZOCR</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>One-Time Capital / Dev Build Cost</t>
-        </is>
-      </c>
-      <c r="C20" s="11" t="n">
-        <v>250000</v>
+          <t>Baseline Zero-Touch Onboarding Rate</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="n">
+        <v>0.22</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>% rate</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
@@ -1191,7 +1194,7 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>1 Senior Fullstack/AI Eng for 1 month</t>
+          <t>Candidate estimate of status quo onboarding completion</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -1203,30 +1206,30 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>TOOLING_MONTHLY</t>
+          <t>TARGET_ZOCR_DAY90</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Monthly Observability Tooling Cost</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="n">
-        <v>15000</v>
+          <t>Target Zero-Touch Onboarding Rate (Day 90)</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="n">
+        <v>0.33</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>INR / mo</t>
+          <t>% rate</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Industry Benchmark</t>
+          <t>Realistic Target</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>LangSmith/Helicone + Datadog APM tier</t>
+          <t>Realistic 90-day trajectory: 22% baseline -&gt; 33% (+11.0% gain)</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
@@ -1238,20 +1241,20 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>ARPU_MONTHLY</t>
+          <t>BUILD_COST</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Average Monthly Subscription Revenue (ARPU)</t>
+          <t>One-Time Capital / Dev Build Cost</t>
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>2999</v>
+        <v>250000</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>INR / biz / mo</t>
+          <t>INR</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
@@ -1261,7 +1264,7 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Cheerio Starter/Growth plan standard SaaS pricing</t>
+          <t>1 Senior Fullstack/AI Eng for 1 month</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1273,20 +1276,20 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>BASE_CHURN</t>
+          <t>TOOLING_MONTHLY</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Baseline Monthly Merchant Churn Rate</t>
-        </is>
-      </c>
-      <c r="C23" s="12" t="n">
-        <v>0.05</v>
+          <t>Monthly Observability Tooling Cost</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>15000</v>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>% / mo</t>
+          <t>INR / mo</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
@@ -1296,7 +1299,7 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>5.0% monthly churn typical in Indian SMB SaaS</t>
+          <t>LangSmith/Helicone + Datadog APM tier</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
@@ -1308,20 +1311,20 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>CHURN_REDUCTION</t>
+          <t>ARPU_MONTHLY</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Estimated Churn Reduction from ZOCR (Base)</t>
-        </is>
-      </c>
-      <c r="C24" s="10" t="n">
-        <v>0.012</v>
+          <t>Average Monthly Subscription Revenue (ARPU)</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="n">
+        <v>2999</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>% absolute</t>
+          <t>INR / biz / mo</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
@@ -1331,7 +1334,7 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>1.2% absolute churn reduction via onboarding fix</t>
+          <t>Cheerio Starter/Growth plan standard SaaS pricing</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
@@ -1343,30 +1346,30 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>META_UTIL_RATE</t>
+          <t>BASE_CHURN</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Meta India Utility Message Delivery Rate</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="n">
-        <v>0.115</v>
+          <t>Baseline Monthly Merchant Churn Rate</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="n">
+        <v>0.05</v>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>INR / msg</t>
+          <t>% / mo</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Verified Meta Doc</t>
+          <t>Industry Benchmark</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>https://developers.facebook.com/docs/whatsapp/pricing</t>
+          <t>5.0% monthly churn typical in Indian SMB SaaS</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
@@ -1378,33 +1381,103 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
+          <t>CHURN_REDUCTION</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Estimated Churn Reduction from ZOCR (Base)</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>% absolute</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Stated Assumption</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>1.2% absolute churn reduction via onboarding fix</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>META_UTIL_RATE</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Meta India Utility Message Delivery Rate</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>INR / msg</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Verified Meta Doc</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>https://developers.facebook.com/docs/whatsapp/pricing</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
           <t>META_MKT_RATE</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Meta India Marketing Message Delivery Rate</t>
         </is>
       </c>
-      <c r="C26" s="8" t="n">
+      <c r="C28" s="8" t="n">
         <v>0.8631</v>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>INR / msg</t>
         </is>
       </c>
-      <c r="E26" s="6" t="inlineStr">
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>Verified Meta Doc</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>https://developers.facebook.com/docs/whatsapp/pricing</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>Oct 2026</t>
         </is>
@@ -1530,11 +1603,11 @@
         </is>
       </c>
       <c r="B7" s="13">
-        <f>Assumptions!C17</f>
+        <f>Assumptions!C18</f>
         <v/>
       </c>
       <c r="C7" s="13">
-        <f>Assumptions!C18</f>
+        <f>Assumptions!C19</f>
         <v/>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -1544,7 +1617,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Assumptions!C17 vs C18</t>
+          <t>Assumptions!C18 vs C19</t>
         </is>
       </c>
     </row>
@@ -1555,11 +1628,11 @@
         </is>
       </c>
       <c r="B8" s="13">
-        <f>Human_Comparison!B10</f>
+        <f>Human_Comparison!B11</f>
         <v/>
       </c>
       <c r="C8" s="13">
-        <f>Human_Comparison!B16</f>
+        <f>Human_Comparison!B17</f>
         <v/>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -1569,7 +1642,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Human_Comparison!B10 vs B16</t>
+          <t>Human_Comparison!B11 vs B17</t>
         </is>
       </c>
     </row>
@@ -1580,7 +1653,7 @@
         </is>
       </c>
       <c r="B9" s="13">
-        <f>Human_Comparison!B11</f>
+        <f>Human_Comparison!B12</f>
         <v/>
       </c>
       <c r="C9" s="13">
@@ -1594,7 +1667,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Human_Comparison!B11 vs B21</t>
+          <t>Human_Comparison!B12 vs B21</t>
         </is>
       </c>
     </row>
@@ -1605,7 +1678,7 @@
         </is>
       </c>
       <c r="B10" s="13">
-        <f>Human_Comparison!B12</f>
+        <f>Human_Comparison!B13</f>
         <v/>
       </c>
       <c r="C10" s="13">
@@ -1619,7 +1692,7 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Human_Comparison!B12 vs B22</t>
+          <t>Human_Comparison!B13 vs B22</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1730,7 @@
         <v>0</v>
       </c>
       <c r="C12" s="13">
-        <f>Assumptions!C21</f>
+        <f>Assumptions!C23</f>
         <v/>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1667,7 +1740,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Assumptions!C21 (LangSmith / Datadog)</t>
+          <t>Assumptions!C23 (LangSmith / Datadog)</t>
         </is>
       </c>
     </row>
@@ -1705,7 +1778,7 @@
         <v>0</v>
       </c>
       <c r="C14" s="13">
-        <f>Assumptions!C20</f>
+        <f>Assumptions!C22</f>
         <v/>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -1715,7 +1788,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Assumptions!C20 (1 Eng for 1 Month)</t>
+          <t>Assumptions!C22 (1 Eng for 1 Month)</t>
         </is>
       </c>
     </row>
@@ -1731,7 +1804,7 @@
         </is>
       </c>
       <c r="C15" s="13">
-        <f>ROUND(Assumptions!C20/Human_Comparison!B25, 2)</f>
+        <f>ROUND(Assumptions!C22/Human_Comparison!B25, 2)</f>
         <v/>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -1882,7 +1955,7 @@
         </is>
       </c>
       <c r="B6" s="18">
-        <f>Assumptions!C6</f>
+        <f>Assumptions!C7</f>
         <v/>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -1892,7 +1965,7 @@
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Assumptions!C6 (Blended across onboarding &amp; mature accounts)</t>
+          <t>Assumptions!C7 (Blended across onboarding &amp; mature accounts)</t>
         </is>
       </c>
     </row>
@@ -1913,7 +1986,7 @@
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>17,500 total queries across all support channels</t>
+          <t>Total monthly inbound volume (17,500 queries)</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1997,7 @@
         </is>
       </c>
       <c r="B8" s="20">
-        <f>Assumptions!C17</f>
+        <f>Assumptions!C18</f>
         <v/>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -1934,7 +2007,7 @@
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>Assumptions!C17 (Status quo static FAQ deflection)</t>
+          <t>Assumptions!C18 (Status quo static FAQ deflection)</t>
         </is>
       </c>
     </row>
@@ -1945,7 +2018,7 @@
         </is>
       </c>
       <c r="B9" s="20">
-        <f>Assumptions!C18</f>
+        <f>Assumptions!C19</f>
         <v/>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -1955,7 +2028,7 @@
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Assumptions!C18 (65% target across top 5 bottlenecks)</t>
+          <t>Assumptions!C19 (65% target across top bottlenecks)</t>
         </is>
       </c>
     </row>
@@ -1974,9 +2047,10 @@
           <t>Queries / mo</t>
         </is>
       </c>
-      <c r="D10" s="19">
-        <f> 17,500 * 65% = 11,375 queries without human rep</f>
-        <v/>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Calc: 17,500 * 65% = 11,375 queries without human rep</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -1994,9 +2068,10 @@
           <t>Queries / mo</t>
         </is>
       </c>
-      <c r="D11" s="19">
-        <f> 17,500 - 11,375 = 6,125 escalated queries</f>
-        <v/>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>Calc: 17,500 - 11,375 = 6,125 escalated queries</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2085,7 +2160,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>Assumptions!C7</f>
+        <f>Assumptions!C8</f>
         <v/>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -2095,7 +2170,7 @@
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Assumptions!C7 (RBI reference rate)</t>
+          <t>Assumptions!C8 (RBI reference rate)</t>
         </is>
       </c>
     </row>
@@ -2106,7 +2181,7 @@
         </is>
       </c>
       <c r="B7" s="22">
-        <f>Assumptions!C8</f>
+        <f>Assumptions!C9</f>
         <v/>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -2116,7 +2191,7 @@
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Assumptions!C8 (openai.com/api/pricing)</t>
+          <t>Assumptions!C9 (openai.com/api/pricing)</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2202,7 @@
         </is>
       </c>
       <c r="B8" s="22">
-        <f>Assumptions!C10</f>
+        <f>Assumptions!C11</f>
         <v/>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -2137,7 +2212,7 @@
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>Assumptions!C10 (openai.com/api/pricing)</t>
+          <t>Assumptions!C11 (openai.com/api/pricing)</t>
         </is>
       </c>
     </row>
@@ -2148,7 +2223,7 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>Assumptions!C11</f>
+        <f>Assumptions!C12</f>
         <v/>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -2158,7 +2233,7 @@
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Assumptions!C11 (Prompt 1k + error 500 + 3 turns 1k)</t>
+          <t>Assumptions!C12 (Prompt 1k + error 500 + 3 turns 1k)</t>
         </is>
       </c>
     </row>
@@ -2169,7 +2244,7 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>Assumptions!C12</f>
+        <f>Assumptions!C13</f>
         <v/>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -2179,7 +2254,7 @@
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Assumptions!C12 (Remediation payload)</t>
+          <t>Assumptions!C13 (Remediation payload)</t>
         </is>
       </c>
     </row>
@@ -2198,9 +2273,10 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="D11" s="19">
-        <f> (Tokens / 1M) * Input Rate</f>
-        <v/>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>Calc: (Tokens / 1M) * Input Rate</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -2218,9 +2294,10 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="D12" s="19">
-        <f> (Tokens / 1M) * Output Rate</f>
-        <v/>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Calc: (Tokens / 1M) * Output Rate</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -2238,9 +2315,10 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="D13" s="19">
-        <f> Input Cost + Output Cost</f>
-        <v/>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>Calc: Input Cost + Output Cost</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -2271,7 +2349,7 @@
         </is>
       </c>
       <c r="B15" s="23">
-        <f>Assumptions!C13</f>
+        <f>Assumptions!C14</f>
         <v/>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -2281,7 +2359,7 @@
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Assumptions!C13 (Edge worker execution + Redis cache)</t>
+          <t>Assumptions!C14 (Edge worker execution + Redis cache)</t>
         </is>
       </c>
     </row>
@@ -2342,9 +2420,10 @@
           <t>INR / mo</t>
         </is>
       </c>
-      <c r="D18" s="19">
-        <f> 17,500 queries * ₹0.20 = ₹3,500 / month</f>
-        <v/>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>Calc: 17,500 queries * ₹0.20 = ₹3,500 / month</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -2362,9 +2441,10 @@
           <t>INR / biz / mo</t>
         </is>
       </c>
-      <c r="D19" s="19">
-        <f> ₹3,500 / 5,000 = ₹0.70 / merchant / month</f>
-        <v/>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>Calc: ₹3,500 / 5,000 = ₹0.70 / merchant / month</t>
+        </is>
       </c>
     </row>
     <row r="20"/>
@@ -2472,7 +2552,7 @@
     <col width="92" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="64" customWidth="1" min="4" max="4"/>
+    <col width="68" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="27" customWidth="1" min="6" max="6"/>
   </cols>
@@ -2521,7 +2601,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>Assumptions!C14</f>
+        <f>Assumptions!C15</f>
         <v/>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -2531,7 +2611,7 @@
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>Assumptions!C14 (Glassdoor/AmbitionBox CS rep benchmark)</t>
+          <t>Assumptions!C15 (Glassdoor/AmbitionBox CS rep benchmark)</t>
         </is>
       </c>
     </row>
@@ -2542,7 +2622,7 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>Assumptions!C15</f>
+        <f>Assumptions!C16</f>
         <v/>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -2552,7 +2632,7 @@
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Assumptions!C15 (Standard 5-day work week)</t>
+          <t>Assumptions!C16 (Standard 5-day work week)</t>
         </is>
       </c>
     </row>
@@ -2563,7 +2643,7 @@
         </is>
       </c>
       <c r="B7" s="18">
-        <f>Assumptions!C16</f>
+        <f>Assumptions!C17</f>
         <v/>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -2573,7 +2653,7 @@
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Assumptions!C16 (Standard chat/ticket handling capacity)</t>
+          <t>Assumptions!C17 (Standard chat/ticket handling capacity)</t>
         </is>
       </c>
     </row>
@@ -2584,7 +2664,7 @@
         </is>
       </c>
       <c r="B8" s="18">
-        <f>B5*B6</f>
+        <f>B6*B7</f>
         <v/>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -2592,9 +2672,10 @@
           <t>Tickets / mo</t>
         </is>
       </c>
-      <c r="D8" s="19">
-        <f> 22 days * 40 tickets/day = 880 tickets / rep / mo</f>
-        <v/>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>Calc: 22 days * 40 tickets/day = 880 tickets / rep / mo</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -2624,7 +2705,7 @@
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>17,500 total queries</t>
+          <t>17,500 total inbound queries</t>
         </is>
       </c>
     </row>
@@ -2643,9 +2724,10 @@
           <t>Agents</t>
         </is>
       </c>
-      <c r="D11" s="19">
-        <f> ROUNDUP(17,500 / 880) = 20 Agents needed to maintain SLA</f>
-        <v/>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>Calc: ROUNDUP(17,500 / 880) = 20 Agents needed</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -2663,9 +2745,10 @@
           <t>INR / mo</t>
         </is>
       </c>
-      <c r="D12" s="19">
-        <f> 20 agents * ₹35,000/mo = ₹7,00,000 / month</f>
-        <v/>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Calc: 20 agents * ₹35,000/mo = ₹7,00,000 / month</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -2683,9 +2766,10 @@
           <t>INR / ticket</t>
         </is>
       </c>
-      <c r="D13" s="19">
-        <f> ₹7,00,000 / 17,500 = ₹40.00 / ticket</f>
-        <v/>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>Calc: ₹7,00,000 / 17,500 = ₹40.00 / ticket</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -2755,9 +2839,10 @@
           <t>Agents</t>
         </is>
       </c>
-      <c r="D17" s="19">
-        <f> ROUNDUP(6,125 / 880) = 7 Agents required</f>
-        <v/>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>Calc: ROUNDUP(6,125 / 880) = 7 Agents required</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -2775,9 +2860,10 @@
           <t>INR / mo</t>
         </is>
       </c>
-      <c r="D18" s="19">
-        <f> 7 agents * ₹35,000/mo = ₹2,45,000 / month</f>
-        <v/>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>Calc: 7 agents * ₹35,000/mo = ₹2,45,000 / month</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -2808,7 +2894,7 @@
         </is>
       </c>
       <c r="B20" s="21">
-        <f>Assumptions!C21</f>
+        <f>Assumptions!C23</f>
         <v/>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -2818,7 +2904,7 @@
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>Assumptions!C21 (LangSmith / Datadog APM = ₹15,000)</t>
+          <t>Assumptions!C23 (LangSmith / Datadog APM = ₹15,000)</t>
         </is>
       </c>
     </row>
@@ -2837,9 +2923,10 @@
           <t>INR / mo</t>
         </is>
       </c>
-      <c r="D21" s="19">
-        <f> ₹2,45,000 salary + ₹3,500 AI + ₹15,000 tooling = ₹2,63,500</f>
-        <v/>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>Calc: ₹2,45,000 salary + ₹3,500 AI + ₹15,000 tooling = ₹2,63,500</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -2857,9 +2944,10 @@
           <t>INR / ticket</t>
         </is>
       </c>
-      <c r="D22" s="19">
-        <f> ₹2,63,500 / 17,500 = ₹15.06 / ticket</f>
-        <v/>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>Calc: ₹2,63,500 / 17,500 = ₹15.06 / ticket</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -2887,9 +2975,10 @@
           <t>Agents</t>
         </is>
       </c>
-      <c r="D24" s="19">
-        <f> 20 agents - 7 agents = 13 agents avoided</f>
-        <v/>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>Calc: 20 agents - 7 agents = 13 agents avoided</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -2907,9 +2996,10 @@
           <t>INR / mo</t>
         </is>
       </c>
-      <c r="D25" s="19">
-        <f> ₹7,00,000 - ₹2,63,500 = ₹4,36,500 / month</f>
-        <v/>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>Calc: ₹7,00,000 - ₹2,63,500 = ₹4,36,500 / month</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -2927,9 +3017,10 @@
           <t>INR / yr</t>
         </is>
       </c>
-      <c r="D26" s="19">
-        <f> ₹4,36,500 * 12 = ₹52.38 Lakhs / year</f>
-        <v/>
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>Calc: ₹4,36,500 * 12 = ₹52.38 Lakhs / year</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -2939,7 +3030,7 @@
         </is>
       </c>
       <c r="B27" s="21">
-        <f>Assumptions!C20</f>
+        <f>Assumptions!C22</f>
         <v/>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -2949,7 +3040,7 @@
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Assumptions!C20 (₹2,50,000 dev build cost)</t>
+          <t>Assumptions!C22 (₹2,50,000 dev build cost)</t>
         </is>
       </c>
     </row>
@@ -2968,9 +3059,10 @@
           <t>Months</t>
         </is>
       </c>
-      <c r="D28" s="19">
-        <f> ₹2,50,000 / ₹4,36,500 = 0.57 Months (~17 Days)</f>
-        <v/>
+      <c r="D28" s="19" t="inlineStr">
+        <is>
+          <t>Calc: ₹2,50,000 / ₹4,36,500 = 0.57 Months (~17 Days)</t>
+        </is>
       </c>
     </row>
     <row r="29"/>
@@ -3109,7 +3201,7 @@
     <col width="65" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="65" customWidth="1" min="4" max="4"/>
+    <col width="69" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
@@ -3179,7 +3271,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>Assumptions!C22</f>
+        <f>Assumptions!C24</f>
         <v/>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -3189,7 +3281,7 @@
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Assumptions!C22 (₹2,999 / month standard tier)</t>
+          <t>Assumptions!C24 (₹2,999 / month standard tier)</t>
         </is>
       </c>
     </row>
@@ -3208,9 +3300,10 @@
           <t>INR / mo</t>
         </is>
       </c>
-      <c r="D7" s="19">
-        <f> 5,000 * ₹2,999 = ₹1,49,95,000 / month (~₹1.50 Cr)</f>
-        <v/>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>Calc: 5,000 * ₹2,999 = ₹1,49,95,000 / month (~₹1.50 Cr)</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -3220,7 +3313,7 @@
         </is>
       </c>
       <c r="B8" s="20">
-        <f>Assumptions!C23</f>
+        <f>Assumptions!C25</f>
         <v/>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -3230,7 +3323,7 @@
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>Assumptions!C23 (5.0% monthly SMB churn benchmark)</t>
+          <t>Assumptions!C25 (5.0% monthly SMB churn benchmark)</t>
         </is>
       </c>
     </row>
@@ -3249,9 +3342,10 @@
           <t>Businesses / mo</t>
         </is>
       </c>
-      <c r="D9" s="19">
-        <f> 5,000 * 5% = 250 merchants lost each month</f>
-        <v/>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>Calc: 5,000 * 5% = 250 merchants lost each month</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -3261,7 +3355,7 @@
         </is>
       </c>
       <c r="B10" s="20">
-        <f>Assumptions!C24</f>
+        <f>Assumptions!C26</f>
         <v/>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -3271,7 +3365,7 @@
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>Assumptions!C24 (1.2% saved by fixing onboarding drop-offs)</t>
+          <t>Assumptions!C26 (1.2% saved by fixing onboarding drop-offs)</t>
         </is>
       </c>
     </row>
@@ -3290,9 +3384,10 @@
           <t>Businesses / mo</t>
         </is>
       </c>
-      <c r="D11" s="19">
-        <f> 5,000 * 1.2% = 60 merchants retained every month</f>
-        <v/>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>Calc: 5,000 * 1.2% = 60 merchants retained every month</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -3310,9 +3405,10 @@
           <t>INR / mo</t>
         </is>
       </c>
-      <c r="D12" s="19">
-        <f> 60 merchants * ₹2,999 = ₹1,79,940 / month</f>
-        <v/>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Calc: 60 merchants * ₹2,999 = ₹1,79,940 / month</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -3330,9 +3426,10 @@
           <t>INR / yr</t>
         </is>
       </c>
-      <c r="D13" s="19">
-        <f> ₹1,79,940 * 12 = ₹21.59 Lakhs / year</f>
-        <v/>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>Calc: ₹1,79,940 * 12 = ₹21.59 Lakhs / year</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -3371,9 +3468,10 @@
           <t>INR / mo</t>
         </is>
       </c>
-      <c r="D15" s="19">
-        <f> Gross Preserved MRR - AI Spend = ₹1,76,440 / month</f>
-        <v/>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>Calc: Gross Preserved MRR - AI Spend = ₹1,76,440 / month</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -3391,9 +3489,10 @@
           <t>x Return</t>
         </is>
       </c>
-      <c r="D16" s="19">
-        <f> Gross Preserved MRR / AI Spend = ₹1,79,940 / ₹3,500 = 51.4x</f>
-        <v/>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>Calc: Gross Preserved MRR / AI Spend = ₹1,79,940 / ₹3,500 = 51.4x</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -3411,9 +3510,10 @@
           <t>x Return</t>
         </is>
       </c>
-      <c r="D17" s="19">
-        <f> Net Retained MRR / AI Spend = ₹1,76,440 / ₹3,500 = 50.4x</f>
-        <v/>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>Calc: Net Retained MRR / AI Spend = ₹1,76,440 / ₹3,500 = 50.4x</t>
+        </is>
       </c>
     </row>
     <row r="18"/>
@@ -3546,15 +3646,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="69" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="53" customWidth="1" min="3" max="3"/>
+    <col width="77" customWidth="1" min="1" max="1"/>
+    <col width="51" customWidth="1" min="2" max="2"/>
+    <col width="69" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="83" customWidth="1" min="6" max="6"/>
+    <col width="89" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3567,7 +3667,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Evaluates 4 Pricing Models with Fully Loaded Unit Costs &amp; Margins</t>
+          <t>Recommends Free Core Co-Pilot + ₹499/mo Priority Add-on • Linked Formulas</t>
         </is>
       </c>
     </row>
@@ -3600,14 +3700,14 @@
       </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>Strategic Fit &amp; Recommendation</t>
+          <t>Strategic Fit &amp; Value Rationale</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Model 1: 100% Free Core Feature (Recommended)</t>
+          <t>Model 1: Free Core Co-Pilot (Recommended Base)</t>
         </is>
       </c>
       <c r="B5" s="33" t="n">
@@ -3618,36 +3718,38 @@
           <t>Free for all active merchants</t>
         </is>
       </c>
-      <c r="D5" s="33" t="n">
-        <v>6.26</v>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="D5" s="26">
+        <f>B15</f>
+        <v/>
+      </c>
+      <c r="E5" s="34" t="inlineStr">
         <is>
           <t>Subsidized</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Maximizes onboarding completion &amp; retention. Subsidized by 50.4x Retention ROI.</t>
+          <t>Maximizes onboarding completion. Net surplus: ₹1.58L/mo (Retention MRR less AI cost).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Model 2: Per-Resolution Micro-Fee</t>
-        </is>
-      </c>
-      <c r="B6" s="33" t="n">
-        <v>5</v>
+          <t>Model 2: Priority Support Add-on (Recommended Upsell)</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="n">
+        <v>499</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Per resolved troubleshooting workflow</t>
-        </is>
-      </c>
-      <c r="D6" s="33" t="n">
-        <v>0.3</v>
+          <t>Per merchant / month</t>
+        </is>
+      </c>
+      <c r="D6" s="26">
+        <f>ROUND((B15*5)+15, 2)</f>
+        <v/>
       </c>
       <c r="E6" s="12">
         <f>ROUND((B6-D6)/B6, 3)</f>
@@ -3655,26 +3757,27 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Friction for SMBs; disincentivizes self-service and causes support backlash.</t>
+          <t>Premium SLA (&lt;15m), dedicated WhatsApp agent. Gross margin: +95.8% via formulas.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Model 3: Prepaid AI Credits Pack</t>
-        </is>
-      </c>
-      <c r="B7" s="26" t="n">
-        <v>199</v>
+          <t>Model 3: Per-Resolution Micro-Fee</t>
+        </is>
+      </c>
+      <c r="B7" s="33" t="n">
+        <v>5</v>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Pack of 50 AI resolutions (₹3.98/res)</t>
-        </is>
-      </c>
-      <c r="D7" s="33" t="n">
-        <v>15</v>
+          <t>Per resolved troubleshooting workflow</t>
+        </is>
+      </c>
+      <c r="D7" s="26">
+        <f>B15</f>
+        <v/>
       </c>
       <c r="E7" s="12">
         <f>ROUND((B7-D7)/B7, 3)</f>
@@ -3682,26 +3785,27 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>High margin (+92.5%), but adds onboarding barrier during crucial activation.</t>
+          <t>High margin (+76.0%), but creates onboarding barrier and causes merchant friction.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Model 4: Premium Dedicated Support Add-On</t>
+          <t>Model 4: Prepaid AI Resolution Pack</t>
         </is>
       </c>
       <c r="B8" s="26" t="n">
-        <v>499</v>
+        <v>199</v>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Per business / month (Unlimited AI + Priority)</t>
-        </is>
-      </c>
-      <c r="D8" s="33" t="n">
-        <v>22.5</v>
+          <t>Pack of 50 AI resolutions (₹3.98/res)</t>
+        </is>
+      </c>
+      <c r="D8" s="26">
+        <f>B15*50</f>
+        <v/>
       </c>
       <c r="E8" s="12">
         <f>ROUND((B8-D8)/B8, 3)</f>
@@ -3709,7 +3813,7 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Viable for high-volume enterprise senders; 95.5% margin, optional add-on.</t>
+          <t>High gross margin (+69.8%), but adds wallet friction during crucial Day 1 onboarding.</t>
         </is>
       </c>
     </row>
@@ -3718,7 +3822,7 @@
     <row r="11">
       <c r="A11" s="24" t="inlineStr">
         <is>
-          <t>FULLY LOADED COST PER RESOLUTION BREAKDOWN (₹)</t>
+          <t>FULLY LOADED AI OPERATIONAL COST PER QUERY (₹) - NO DOUBLE COUNTING</t>
         </is>
       </c>
     </row>
@@ -3728,57 +3832,77 @@
           <t>LLM Token Inference (GPT-4o-mini blended)</t>
         </is>
       </c>
-      <c r="B12" s="34" t="n">
-        <v>0.2</v>
+      <c r="B12" s="35">
+        <f>Token_Economics!B16</f>
+        <v/>
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
-          <t>Token_Economics!B16</t>
+          <t>Token_Economics!B16 (₹0.20 per query)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Observability &amp; Cache Overhead (LangSmith + Redis)</t>
-        </is>
-      </c>
-      <c r="B13" s="34" t="n">
-        <v>0.1</v>
+          <t>Edge Cache &amp; Serverless Buffer (Cloudflare/Redis)</t>
+        </is>
+      </c>
+      <c r="B13" s="35">
+        <f>Assumptions!C14</f>
+        <v/>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>Allocated tooling buffer</t>
+          <t>Assumptions!C14 (₹0.14 per query)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Amortized Human Escalation Share (across 35% unassisted queries)</t>
-        </is>
-      </c>
-      <c r="B14" s="34" t="n">
-        <v>5.96</v>
-      </c>
-      <c r="C14" s="19">
-        <f>Human_Comparison!B18 / Volume_Model!B7</f>
-        <v/>
+          <t>Observability &amp; Tooling per Query (LangSmith/Datadog)</t>
+        </is>
+      </c>
+      <c r="B14" s="35">
+        <f>ROUND(Assumptions!C23/Volume_Model!B7, 2)</f>
+        <v/>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>Calc: ₹15,000 monthly tooling / 17,500 queries = ₹0.86</t>
+        </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Total Fully Loaded Cost per Support Query (₹)</t>
-        </is>
-      </c>
-      <c r="B15" s="34">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Total Fully Loaded AI Cost per Query (₹)</t>
+        </is>
+      </c>
+      <c r="B15" s="35">
         <f>B12+B13+B14</f>
         <v/>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>Complete blended operational cost per interaction</t>
+          <t>Calc: Direct operational running cost for AI Co-Pilot (₹1.20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>SEPARATE OPERATIONAL LINE: Amortized Human Escalation Share</t>
+        </is>
+      </c>
+      <c r="B16" s="35">
+        <f>ROUND(Human_Comparison!B18/Volume_Model!B7, 2)</f>
+        <v/>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>Calc: ₹2,45,000 human escalation salary / 17,500 queries = ₹14.00</t>
         </is>
       </c>
     </row>
@@ -3793,14 +3917,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="63" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="77" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3856,7 +3980,7 @@
           <t>&gt; 2x Baseline (&gt; ₹0.40 / query)</t>
         </is>
       </c>
-      <c r="C5" s="35" t="inlineStr">
+      <c r="C5" s="36" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3883,7 +4007,7 @@
           <t>&gt; 140% 7-day rolling avg (&gt; 4,200 tokens)</t>
         </is>
       </c>
-      <c r="C6" s="36" t="inlineStr">
+      <c r="C6" s="37" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3910,7 +4034,7 @@
           <t>&gt; 50 sessions / 24 hours</t>
         </is>
       </c>
-      <c r="C7" s="35" t="inlineStr">
+      <c r="C7" s="36" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3922,14 +4046,14 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Throttle merchant rate limit; trigger white-glove onboarding call</t>
+          <t>Throttle merchant rate limit; trigger proactive white-glove onboarding check</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Zero-Touch Deflection Rate (ZOCR)</t>
+          <t>Deflection Rate (7-day verified)</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -3937,7 +4061,7 @@
           <t>&lt; 40% (Target: 65%)</t>
         </is>
       </c>
-      <c r="C8" s="37" t="inlineStr">
+      <c r="C8" s="38" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -3949,59 +4073,86 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Review Meta Cloud API error changes; retrain diagnostic intent embeddings</t>
+          <t>Audit recent Meta Cloud API changelogs; update regex and error intent models</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>7-Day Ticket Reopen Rate</t>
+          <t>Zero-Touch Onboarding Rate (ZOCR)</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>&gt; 5.0% of deflected tickets</t>
-        </is>
-      </c>
-      <c r="C9" s="35" t="inlineStr">
+          <t>&lt; 25% (Target: 33% at Day 90)</t>
+        </is>
+      </c>
+      <c r="C9" s="36" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>QA Lead / Support Lead</t>
+          <t>Onboarding &amp; Growth Lead</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Audit auto-fix false positives; refine pre-flight regex linter rules</t>
+          <t>Review Day 1-7 drop-off funnels; inspect WABA phone binding failure logs</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
+          <t>7-Day Ticket Reopen Rate</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>&gt; 5.0% of deflected tickets</t>
+        </is>
+      </c>
+      <c r="C10" s="36" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>QA Lead / Support Lead</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Audit auto-fix false positives; refine pre-flight regex linter rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
           <t>Monthly Token Invoice Reconciliation</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>OpenAI invoice vs logs variance &gt; ±2%</t>
         </is>
       </c>
-      <c r="C10" s="36" t="inlineStr">
+      <c r="C11" s="37" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Finance / Eng Lead</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Reconcile dropped webhooks, orphaned sessions, or billing discrepancies</t>
         </is>

</xml_diff>

<commit_message>
Comprehensive polish: dual-base ROI reconciliation, 4 scenario screenshots, rollback support, and candidate reflection
</commit_message>
<xml_diff>
--- a/cheerio/assignment/cheerio_cost_model.xlsx
+++ b/cheerio/assignment/cheerio_cost_model.xlsx
@@ -1494,14 +1494,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="82" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="51" customWidth="1" min="3" max="3"/>
     <col width="29" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="57" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1821,7 +1821,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Gross Merchant Retention ROI</t>
+          <t>Gross Merchant Retention ROI (Direct Tokens)</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
@@ -1830,7 +1830,7 @@
         </is>
       </c>
       <c r="C16" s="13">
-        <f>Retention_ROI!B16</f>
+        <f>Retention_ROI!B18</f>
         <v/>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -1840,14 +1840,14 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Retention_ROI!B16 (Gross MRR / AI Spend)</t>
+          <t>Retention_ROI!B18 (Gross MRR / AI Tokens)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>Net Merchant Retention ROI</t>
+          <t>Net Merchant Retention ROI (Direct Tokens)</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
@@ -1856,7 +1856,7 @@
         </is>
       </c>
       <c r="C17" s="15">
-        <f>Retention_ROI!B17</f>
+        <f>Retention_ROI!B19</f>
         <v/>
       </c>
       <c r="D17" s="14" t="inlineStr">
@@ -1866,7 +1866,33 @@
       </c>
       <c r="E17" s="16" t="inlineStr">
         <is>
-          <t>Retention_ROI!B17 (Net MRR / AI Spend)</t>
+          <t>Retention_ROI!B19 (Net MRR / AI Tokens)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Net Merchant Retention ROI (Total Program)</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C18" s="13">
+        <f>Retention_ROI!B21</f>
+        <v/>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>8.7x Return</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Retention_ROI!B21 (Net MRR / ₹18.5k Total AI+Tooling)</t>
         </is>
       </c>
     </row>
@@ -3195,15 +3221,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="65" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="69" customWidth="1" min="4" max="4"/>
+    <col width="74" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3435,7 +3463,7 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Monthly Cheerio Co-Pilot AI Token Cost (₹)</t>
+          <t>Direct Monthly AI Token Cost (₹)</t>
         </is>
       </c>
       <c r="B14" s="21">
@@ -3449,18 +3477,18 @@
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>Token_Economics!B18 (₹3,500 total monthly AI spend)</t>
+          <t>Token_Economics!B18 (₹3,500 direct LLM API spend)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Net Monthly Retained Financial Value (₹)</t>
+          <t>Total Monthly Program Cost (Tokens + Tooling) (₹)</t>
         </is>
       </c>
       <c r="B15" s="21">
-        <f>B12-B14</f>
+        <f>Human_Comparison!B20</f>
         <v/>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -3470,168 +3498,285 @@
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Calc: Gross Preserved MRR - AI Spend = ₹1,76,440 / month</t>
+          <t>Human_Comparison!B20 (₹3,500 tokens + ₹15,000 Redis/observability)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Gross ROI on AI Spend</t>
-        </is>
-      </c>
-      <c r="B16" s="31">
-        <f>ROUND(B12/B14, 1)</f>
+          <t>Net Monthly Preserved MRR (vs Direct Tokens) (₹)</t>
+        </is>
+      </c>
+      <c r="B16" s="21">
+        <f>B12-B14</f>
         <v/>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>x Return</t>
+          <t>INR / mo</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>Calc: Gross Preserved MRR / AI Spend = ₹1,79,940 / ₹3,500 = 51.4x</t>
+          <t>Calc: Gross Preserved MRR - Direct Token Spend = ₹1,76,440 / mo</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Net ROI on AI Spend</t>
-        </is>
-      </c>
-      <c r="B17" s="31">
-        <f>ROUND(B15/B14, 1)</f>
+          <t>Net Monthly Preserved MRR (vs Total Program Cost) (₹)</t>
+        </is>
+      </c>
+      <c r="B17" s="21">
+        <f>B12-B15</f>
         <v/>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
+          <t>INR / mo</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>Calc: Gross Preserved MRR - Total Program Cost = ₹1,61,440 / mo</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Gross ROI Multiple on Direct Token Spend</t>
+        </is>
+      </c>
+      <c r="B18" s="31">
+        <f>ROUND(B12/B14, 1)</f>
+        <v/>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
           <t>x Return</t>
         </is>
       </c>
-      <c r="D17" s="19" t="inlineStr">
-        <is>
-          <t>Calc: Net Retained MRR / AI Spend = ₹1,76,440 / ₹3,500 = 50.4x</t>
-        </is>
-      </c>
-    </row>
-    <row r="18"/>
-    <row r="19"/>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>Calc: Gross Preserved MRR / Direct Tokens = ₹1,79,940 / ₹3,500 = 51.4x</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Net ROI Multiple on Direct Token Spend</t>
+        </is>
+      </c>
+      <c r="B19" s="31">
+        <f>ROUND(B16/B14, 1)</f>
+        <v/>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>x Return</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>Calc: Net Preserved MRR / Direct Tokens = ₹1,76,440 / ₹3,500 = 50.4x</t>
+        </is>
+      </c>
+    </row>
     <row r="20">
-      <c r="A20" s="24" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Gross ROI Multiple on Total Program Cost</t>
+        </is>
+      </c>
+      <c r="B20" s="31">
+        <f>ROUND(B12/B15, 1)</f>
+        <v/>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>x Return</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>Calc: Gross Preserved MRR / Total Program = ₹1,79,940 / ₹18,500 = 9.7x</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Net ROI Multiple on Total Program Cost</t>
+        </is>
+      </c>
+      <c r="B21" s="31">
+        <f>ROUND(B17/B15, 1)</f>
+        <v/>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>x Return</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>Calc: Net Preserved MRR / Total Program = ₹1,61,440 / ₹18,500 = 8.7x</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="24" t="inlineStr">
         <is>
           <t>CHURN REDUCTION SENSITIVITY TABLE (Low / Base / High)</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="25" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="25" t="inlineStr">
         <is>
           <t>Scenario</t>
         </is>
       </c>
-      <c r="B21" s="25" t="inlineStr">
+      <c r="B24" s="25" t="inlineStr">
         <is>
           <t>Absolute Churn Reduction</t>
         </is>
       </c>
-      <c r="C21" s="25" t="inlineStr">
+      <c r="C24" s="25" t="inlineStr">
         <is>
           <t>Retained Merchants/Mo</t>
         </is>
       </c>
-      <c r="D21" s="25" t="inlineStr">
+      <c r="D24" s="25" t="inlineStr">
         <is>
           <t>Gross Preserved MRR (₹)</t>
         </is>
       </c>
-      <c r="E21" s="25" t="inlineStr">
-        <is>
-          <t>Net Preserved MRR (₹)</t>
-        </is>
-      </c>
-      <c r="F21" s="25" t="inlineStr">
-        <is>
-          <t>Net ROI Multiple</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="E24" s="25" t="inlineStr">
+        <is>
+          <t>Net MRR vs Tokens (₹)</t>
+        </is>
+      </c>
+      <c r="F24" s="25" t="inlineStr">
+        <is>
+          <t>Net ROI (Tokens)</t>
+        </is>
+      </c>
+      <c r="G24" s="25" t="inlineStr">
+        <is>
+          <t>Net MRR vs Total Spend (₹)</t>
+        </is>
+      </c>
+      <c r="H24" s="25" t="inlineStr">
+        <is>
+          <t>Net ROI (Total Spend)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Conservative (Low)</t>
         </is>
       </c>
-      <c r="B22" s="29" t="n">
+      <c r="B25" s="29" t="n">
         <v>0.005</v>
       </c>
-      <c r="C22" s="30">
-        <f>ROUND(5000*B22,0)</f>
-        <v/>
-      </c>
-      <c r="D22" s="26">
-        <f>C22*2999</f>
-        <v/>
-      </c>
-      <c r="E22" s="26">
-        <f>D22-3500</f>
-        <v/>
-      </c>
-      <c r="F22" s="32">
-        <f>ROUND(E22/3500,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="C25" s="30">
+        <f>ROUND(5000*B25,0)</f>
+        <v/>
+      </c>
+      <c r="D25" s="26">
+        <f>C25*2999</f>
+        <v/>
+      </c>
+      <c r="E25" s="26">
+        <f>D25-3500</f>
+        <v/>
+      </c>
+      <c r="F25" s="32">
+        <f>ROUND(E25/3500,1)</f>
+        <v/>
+      </c>
+      <c r="G25" s="26">
+        <f>D25-18500</f>
+        <v/>
+      </c>
+      <c r="H25" s="32">
+        <f>ROUND(G25/18500,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Expected (Base)</t>
         </is>
       </c>
-      <c r="B23" s="29" t="n">
+      <c r="B26" s="29" t="n">
         <v>0.012</v>
       </c>
-      <c r="C23" s="30">
-        <f>ROUND(5000*B23,0)</f>
-        <v/>
-      </c>
-      <c r="D23" s="26">
-        <f>C23*2999</f>
-        <v/>
-      </c>
-      <c r="E23" s="26">
-        <f>D23-3500</f>
-        <v/>
-      </c>
-      <c r="F23" s="32">
-        <f>ROUND(E23/3500,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="C26" s="30">
+        <f>ROUND(5000*B26,0)</f>
+        <v/>
+      </c>
+      <c r="D26" s="26">
+        <f>C26*2999</f>
+        <v/>
+      </c>
+      <c r="E26" s="26">
+        <f>D26-3500</f>
+        <v/>
+      </c>
+      <c r="F26" s="32">
+        <f>ROUND(E26/3500,1)</f>
+        <v/>
+      </c>
+      <c r="G26" s="26">
+        <f>D26-18500</f>
+        <v/>
+      </c>
+      <c r="H26" s="32">
+        <f>ROUND(G26/18500,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>Aggressive (High)</t>
         </is>
       </c>
-      <c r="B24" s="29" t="n">
+      <c r="B27" s="29" t="n">
         <v>0.02</v>
       </c>
-      <c r="C24" s="30">
-        <f>ROUND(5000*B24,0)</f>
-        <v/>
-      </c>
-      <c r="D24" s="26">
-        <f>C24*2999</f>
-        <v/>
-      </c>
-      <c r="E24" s="26">
-        <f>D24-3500</f>
-        <v/>
-      </c>
-      <c r="F24" s="32">
-        <f>ROUND(E24/3500,1)</f>
+      <c r="C27" s="30">
+        <f>ROUND(5000*B27,0)</f>
+        <v/>
+      </c>
+      <c r="D27" s="26">
+        <f>C27*2999</f>
+        <v/>
+      </c>
+      <c r="E27" s="26">
+        <f>D27-3500</f>
+        <v/>
+      </c>
+      <c r="F27" s="32">
+        <f>ROUND(E27/3500,1)</f>
+        <v/>
+      </c>
+      <c r="G27" s="26">
+        <f>D27-18500</f>
+        <v/>
+      </c>
+      <c r="H27" s="32">
+        <f>ROUND(G27/18500,1)</f>
         <v/>
       </c>
     </row>

</xml_diff>